<commit_message>
long time no commit....
</commit_message>
<xml_diff>
--- a/annotation/Species_list_vs_CATAMI_2025_01.xlsx
+++ b/annotation/Species_list_vs_CATAMI_2025_01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universitytasmania-my.sharepoint.com/personal/jan_jansen_utas_edu_au/Documents/science/SouthernOceanBiodiversityMapping/ARC_Data/annotation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="8_{FD0C8598-491B-401D-B81F-83F6C092F470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A0EC056-56E1-4E3B-A625-398F07ECADBF}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{FD0C8598-491B-401D-B81F-83F6C092F470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{227FD468-569D-4003-B3C7-8EE9ADA145E2}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19950" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21990" yWindow="-20820" windowWidth="38700" windowHeight="19725" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COVER_naming" sheetId="1" r:id="rId1"/>
@@ -2239,6 +2239,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2535,7 +2539,7 @@
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.42578125" customWidth="1"/>
-    <col min="5" max="5" width="50.85546875" customWidth="1"/>
+    <col min="5" max="5" width="83.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="68.42578125" style="11" customWidth="1"/>
     <col min="7" max="7" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.7109375" bestFit="1" customWidth="1"/>
@@ -7861,7 +7865,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="98" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>109</v>
       </c>

</xml_diff>